<commit_message>
project master data added company layer
</commit_message>
<xml_diff>
--- a/template/Project_Template.xlsx
+++ b/template/Project_Template.xlsx
@@ -27,15 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Project Code</t>
   </si>
   <si>
     <t>Project Description</t>
-  </si>
-  <si>
-    <t>Company</t>
   </si>
 </sst>
 </file>
@@ -1005,22 +1002,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="2"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.8296296296296" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:3">
+    <row r="1" ht="15.75" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>